<commit_message>
add emp id on emp list
</commit_message>
<xml_diff>
--- a/src/assets/excel/template-employee.xlsx
+++ b/src/assets/excel/template-employee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gbvh\src\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D50705-ADEC-4B88-9B5D-B82B72F71A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BFA11B-9987-4DDC-99DA-F32BDA4B22C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4D14FBF3-6023-4295-9F6A-24B32DAA4FB2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>ID</t>
   </si>
@@ -61,14 +61,25 @@
   </si>
   <si>
     <t>LABOR_TYPE</t>
+  </si>
+  <si>
+    <t>ID_COMPANY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -84,7 +95,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -92,12 +103,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,51 +440,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC8517A-5AD9-4F8B-8EA0-BFCA706E10C3}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="12" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="13" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="N1" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
validasi excel upload on emp management
</commit_message>
<xml_diff>
--- a/src/assets/excel/template-employee.xlsx
+++ b/src/assets/excel/template-employee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gbvh\src\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91019C2-234E-448E-A4FA-CCEC45A52083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F048E771-0013-433E-B301-823A7564FA7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4D14FBF3-6023-4295-9F6A-24B32DAA4FB2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>ID</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>BPJS_KETENAGAKERJAAN</t>
+  </si>
+  <si>
+    <t>RESIGN_DATE</t>
   </si>
 </sst>
 </file>
@@ -445,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC8517A-5AD9-4F8B-8EA0-BFCA706E10C3}">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -455,15 +458,16 @@
     <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="10.7109375" customWidth="1"/>
-    <col min="14" max="14" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.42578125" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -489,24 +493,27 @@
         <v>10</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>